<commit_message>
spec change: regenerated site risk mapping from SiteRisk_MappingSpec.xlsx
</commit_message>
<xml_diff>
--- a/spec/SiteRisk_MappingSpec.xlsx
+++ b/spec/SiteRisk_MappingSpec.xlsx
@@ -525,7 +525,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -553,7 +552,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -581,7 +579,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -609,7 +606,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -637,7 +633,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -665,7 +660,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -693,7 +687,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -701,7 +694,6 @@
           <t>riskLevel</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>string</t>
@@ -729,7 +721,6 @@
           <t>advisory</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>string</t>
@@ -757,7 +748,6 @@
           <t>dispatchFlag</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>boolean</t>
@@ -844,7 +834,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>aqi &gt;= 150</t>
+          <t>aqi &gt;= 140</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>